<commit_message>
Pruebas e2e de Word/Excel/PowerPoint a PDF y encadenado Word→PDF→EPUB en la app empaquetada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MNQ3cZTHgxewBkKhBCN5vB
</commit_message>
<xml_diff>
--- a/tests/fixtures/office/libro.xlsx
+++ b/tests/fixtures/office/libro.xlsx
@@ -639,6 +639,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -717,6 +719,32 @@
   </sheetPr>
   <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Gráficos de Excel, Word y PowerPoint dibujados en SVG; ecuaciones de Word como texto
Columnas, barras (agrupadas, apiladas, al 100 %), líneas, áreas, sectores, anillos y dispersión,
con título, ejes, rejilla, leyenda y etiquetas de datos. Los gráficos sin datos en caché
(openpyxl, XlsxWriter) se completan leyendo las celdas. En Excel, los gráficos e imágenes se
colocan sobre las celdas en las que están anclados.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MNQ3cZTHgxewBkKhBCN5vB
</commit_message>
<xml_diff>
--- a/tests/fixtures/office/libro.xlsx
+++ b/tests/fixtures/office/libro.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ancha" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gráficos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -192,6 +193,375 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ventas y gastos</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Gráficos'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Gráficos'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Gráficos'!$B$2:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Gráficos'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Gráficos'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Gráficos'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Euros</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Tendencia</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Gráficos'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Gráficos'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Gráficos'!$B$2:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Gráficos'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Gráficos'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Gráficos'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Reparto</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Gráficos'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Gráficos'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Gráficos'!$B$2:$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2304000" cy="2160000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -946,4 +1316,101 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Gastos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ene</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>120</v>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C3" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>90</v>
+      </c>
+      <c r="C4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Abr</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>180</v>
+      </c>
+      <c r="C5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>210</v>
+      </c>
+      <c r="C6" t="n">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>